<commit_message>
Implement unit merge and drag system
- Add UnitDragSystem for drag and drop functionality
- Add UnitMergeManager for unit merging (2 same grade+name → next grade)
- Update UnitPlacementManager with Dictionary-based position tracking
- Add GetUnitAtPosition, MoveUnitToPosition, RemoveUnit, PlaceUnitAtPosition methods
- Update Unit class with mouse drag events (OnMouseDown/Drag/Up)
- Add Uncommon grade to GradeType enum
- Add Instance singleton and GetTowersByGrade to GameDataSO
- Add visual grade colors including Uncommon (light green)
</commit_message>
<xml_diff>
--- a/Assets/Data/GameData.xlsx
+++ b/Assets/Data/GameData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\DefenceGame\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F19E12D4-BBAC-4EA9-9C00-25D5268C10F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5591567E-02E7-4D8C-AF09-A0A6A875B673}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6105" yWindow="2250" windowWidth="21600" windowHeight="11385" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-1260" yWindow="1650" windowWidth="21600" windowHeight="11385" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enemies" sheetId="1" r:id="rId1"/>
@@ -106,9 +106,6 @@
     <t>RangeMultiplier</t>
   </si>
   <si>
-    <t>AttackSpeedMultiplier</t>
-  </si>
-  <si>
     <t>BlackSlime</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -134,6 +131,10 @@
   </si>
   <si>
     <t>Probability</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>AttackSpeedMultiplier</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1115,10 +1116,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="D2">
         <v>1.5</v>
@@ -1132,10 +1133,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C3">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -1149,16 +1150,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C4">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="D4">
         <v>5</v>
       </c>
       <c r="E4">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -1166,10 +1167,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C5">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="D5">
         <v>2</v>
@@ -1183,10 +1184,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6">
-        <v>5000</v>
+        <v>1000</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -1205,6 +1206,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="4" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.25" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -1237,7 +1242,7 @@
         <v>10</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -1263,7 +1268,7 @@
         <v>3</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -1271,19 +1276,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C4">
         <v>50</v>
       </c>
       <c r="D4">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="E4">
         <v>3</v>
       </c>
       <c r="F4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -1297,13 +1302,13 @@
         <v>100</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>3</v>
       </c>
       <c r="F5" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1383,7 +1388,7 @@
         <v>2</v>
       </c>
       <c r="C4">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -1488,7 +1493,7 @@
       </c>
       <c r="C10">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1596,7 +1601,7 @@
       </c>
       <c r="C16">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -1678,7 +1683,7 @@
         <v>8</v>
       </c>
       <c r="B1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -1686,7 +1691,7 @@
         <v>10</v>
       </c>
       <c r="B2">
-        <v>25</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -1694,7 +1699,7 @@
         <v>12</v>
       </c>
       <c r="B3">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -1702,7 +1707,7 @@
         <v>13</v>
       </c>
       <c r="B4">
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -1710,7 +1715,7 @@
         <v>15</v>
       </c>
       <c r="B5">
-        <v>25</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1741,7 +1746,7 @@
         <v>22</v>
       </c>
       <c r="D1" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Fix Unit Drag/Merge System: RareColor visual feedback, same name upgrade merge, drag stability
</commit_message>
<xml_diff>
--- a/Assets/Data/GameData.xlsx
+++ b/Assets/Data/GameData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\DefenceGame\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5591567E-02E7-4D8C-AF09-A0A6A875B673}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29F01C92-90DE-45C3-B2F3-68D2F64EE276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1260" yWindow="1650" windowWidth="21600" windowHeight="11385" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enemies" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="32">
   <si>
     <t>Id</t>
   </si>
@@ -135,6 +135,10 @@
   </si>
   <si>
     <t>AttackSpeedMultiplier</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rare</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1204,10 +1208,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="4" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1309,6 +1314,246 @@
       </c>
       <c r="F5" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6">
+        <v>3</v>
+      </c>
+      <c r="F6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7">
+        <v>25</v>
+      </c>
+      <c r="D7">
+        <v>0.8</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8">
+        <v>50</v>
+      </c>
+      <c r="D8">
+        <v>0.8</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+      <c r="F8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9">
+        <v>100</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>3</v>
+      </c>
+      <c r="F9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10">
+        <v>10</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11">
+        <v>25</v>
+      </c>
+      <c r="D11">
+        <v>0.8</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12">
+        <v>50</v>
+      </c>
+      <c r="D12">
+        <v>0.8</v>
+      </c>
+      <c r="E12">
+        <v>3</v>
+      </c>
+      <c r="F12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13">
+        <v>100</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>3</v>
+      </c>
+      <c r="F13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14">
+        <v>10</v>
+      </c>
+      <c r="D14">
+        <v>2</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15">
+        <v>25</v>
+      </c>
+      <c r="D15">
+        <v>0.8</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+      <c r="F15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16">
+        <v>50</v>
+      </c>
+      <c r="D16">
+        <v>0.8</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17">
+        <v>100</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: Change Length to Count for List<TowerData>
</commit_message>
<xml_diff>
--- a/Assets/Data/GameData.xlsx
+++ b/Assets/Data/GameData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\DefenceGame\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29F01C92-90DE-45C3-B2F3-68D2F64EE276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6C024E7-2542-42F5-8070-2F4E86D37221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enemies" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="33">
   <si>
     <t>Id</t>
   </si>
@@ -139,6 +139,10 @@
   </si>
   <si>
     <t>Rare</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Uncommon</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1208,12 +1212,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="4" width="12.375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -1333,7 +1337,7 @@
         <v>3</v>
       </c>
       <c r="F6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -1353,7 +1357,7 @@
         <v>3</v>
       </c>
       <c r="F7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -1373,7 +1377,7 @@
         <v>3</v>
       </c>
       <c r="F8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -1393,7 +1397,7 @@
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -1413,7 +1417,7 @@
         <v>3</v>
       </c>
       <c r="F10" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -1433,7 +1437,7 @@
         <v>3</v>
       </c>
       <c r="F11" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -1453,7 +1457,7 @@
         <v>3</v>
       </c>
       <c r="F12" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -1473,7 +1477,7 @@
         <v>3</v>
       </c>
       <c r="F13" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -1493,7 +1497,7 @@
         <v>3</v>
       </c>
       <c r="F14" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -1513,7 +1517,7 @@
         <v>3</v>
       </c>
       <c r="F15" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -1533,7 +1537,7 @@
         <v>3</v>
       </c>
       <c r="F16" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -1553,6 +1557,86 @@
         <v>3</v>
       </c>
       <c r="F17" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18">
+        <v>10</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18">
+        <v>3</v>
+      </c>
+      <c r="F18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19">
+        <v>25</v>
+      </c>
+      <c r="D19">
+        <v>0.8</v>
+      </c>
+      <c r="E19">
+        <v>3</v>
+      </c>
+      <c r="F19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20">
+        <v>50</v>
+      </c>
+      <c r="D20">
+        <v>0.8</v>
+      </c>
+      <c r="E20">
+        <v>3</v>
+      </c>
+      <c r="F20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21">
+        <v>100</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <v>3</v>
+      </c>
+      <c r="F21" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1917,9 +2001,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="11.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1936,31 +2021,39 @@
         <v>10</v>
       </c>
       <c r="B2">
-        <v>67</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="B3">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>15</v>
       </c>
-      <c r="B5">
-        <v>3</v>
+      <c r="B6">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1971,10 +2064,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.5" bestFit="1" customWidth="1"/>
@@ -2010,7 +2103,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="B3">
         <v>1.5</v>
@@ -2024,29 +2117,43 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="C4">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D4">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>2.5</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>15</v>
       </c>
-      <c r="B5">
+      <c r="B6">
         <v>5</v>
       </c>
-      <c r="C5">
-        <v>3</v>
-      </c>
-      <c r="D5">
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: Normalize tower IDs (1-20 → 1-4) for 5-tier grade system
</commit_message>
<xml_diff>
--- a/Assets/Data/GameData.xlsx
+++ b/Assets/Data/GameData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\DefenceGame\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6C024E7-2542-42F5-8070-2F4E86D37221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56671290-5FBF-4E6A-B9DC-93BF45949803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enemies" sheetId="1" r:id="rId1"/>
@@ -70,9 +70,6 @@
     <t>Common</t>
   </si>
   <si>
-    <t>Mage</t>
-  </si>
-  <si>
     <t>Rare</t>
   </si>
   <si>
@@ -126,10 +123,6 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>MageTower</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>Probability</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -143,6 +136,14 @@
   </si>
   <si>
     <t>Uncommon</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Wizard</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>WizardTower</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1124,7 +1125,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2">
         <v>30</v>
@@ -1141,7 +1142,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3">
         <v>50</v>
@@ -1158,7 +1159,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4">
         <v>20</v>
@@ -1175,7 +1176,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -1192,7 +1193,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C6">
         <v>1000</v>
@@ -1265,7 +1266,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="C3">
         <v>25</v>
@@ -1285,7 +1286,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C4">
         <v>50</v>
@@ -1305,7 +1306,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -1337,7 +1338,7 @@
         <v>3</v>
       </c>
       <c r="F6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -1345,7 +1346,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="C7">
         <v>25</v>
@@ -1357,7 +1358,7 @@
         <v>3</v>
       </c>
       <c r="F7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -1365,7 +1366,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C8">
         <v>50</v>
@@ -1377,7 +1378,7 @@
         <v>3</v>
       </c>
       <c r="F8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -1385,7 +1386,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9">
         <v>100</v>
@@ -1397,7 +1398,7 @@
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -1417,7 +1418,7 @@
         <v>3</v>
       </c>
       <c r="F10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -1425,7 +1426,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="C11">
         <v>25</v>
@@ -1437,7 +1438,7 @@
         <v>3</v>
       </c>
       <c r="F11" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -1445,7 +1446,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C12">
         <v>50</v>
@@ -1457,7 +1458,7 @@
         <v>3</v>
       </c>
       <c r="F12" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -1465,7 +1466,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C13">
         <v>100</v>
@@ -1477,7 +1478,7 @@
         <v>3</v>
       </c>
       <c r="F13" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -1497,7 +1498,7 @@
         <v>3</v>
       </c>
       <c r="F14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -1505,7 +1506,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="C15">
         <v>25</v>
@@ -1517,7 +1518,7 @@
         <v>3</v>
       </c>
       <c r="F15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -1525,7 +1526,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C16">
         <v>50</v>
@@ -1537,7 +1538,7 @@
         <v>3</v>
       </c>
       <c r="F16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -1545,7 +1546,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C17">
         <v>100</v>
@@ -1557,7 +1558,7 @@
         <v>3</v>
       </c>
       <c r="F17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -1577,7 +1578,7 @@
         <v>3</v>
       </c>
       <c r="F18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -1585,7 +1586,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="C19">
         <v>25</v>
@@ -1597,7 +1598,7 @@
         <v>3</v>
       </c>
       <c r="F19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -1605,7 +1606,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C20">
         <v>50</v>
@@ -1617,7 +1618,7 @@
         <v>3</v>
       </c>
       <c r="F20" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -1625,7 +1626,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C21">
         <v>100</v>
@@ -1637,7 +1638,7 @@
         <v>3</v>
       </c>
       <c r="F21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1660,19 +1661,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>19</v>
-      </c>
-      <c r="E1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -2013,7 +2014,7 @@
         <v>8</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -2026,7 +2027,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B3">
         <v>25</v>
@@ -2034,7 +2035,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <v>12</v>
@@ -2042,7 +2043,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <v>6</v>
@@ -2050,7 +2051,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6">
         <v>2</v>
@@ -2078,13 +2079,13 @@
         <v>8</v>
       </c>
       <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" t="s">
-        <v>22</v>
-      </c>
       <c r="D1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -2103,7 +2104,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B3">
         <v>1.5</v>
@@ -2117,7 +2118,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <v>2</v>
@@ -2131,7 +2132,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <v>2.5</v>
@@ -2145,7 +2146,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6">
         <v>5</v>

</xml_diff>

<commit_message>
Fix tower type names: Wizard->Mage, WizardTower->MageTower
Update TowerLevelManager towerTypes array to match actual unit names
from console logs
</commit_message>
<xml_diff>
--- a/Assets/Data/GameData.xlsx
+++ b/Assets/Data/GameData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\DefenceGame\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56671290-5FBF-4E6A-B9DC-93BF45949803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18E695DA-5EBB-45EB-9F70-82122E2FAA49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enemies" sheetId="1" r:id="rId1"/>
@@ -2022,7 +2022,8 @@
         <v>10</v>
       </c>
       <c r="B2">
-        <v>55</v>
+        <f>100-SUM(B3:B6)</f>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -2030,7 +2031,7 @@
         <v>30</v>
       </c>
       <c r="B3">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -2038,7 +2039,7 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -2046,7 +2047,7 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -2054,7 +2055,7 @@
         <v>14</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Arrow lifetime, damage detection, stats calculation, and folder reorganization
- Fix Archer arrows to destroy after 1 second if not hitting enemy
- Fix arrows to deal damage on enemy collision via OnTriggerEnter2D
- Fix Wizard GroundEffect damage detection with trigger/non-trigger colliders
- Add LevelBonusAttackPower field to TowerData for Excel integration
- Update Unit.Initialize to calculate stats using Excel UnitGrades sheet:
  - AttackPower = (BaseAttack + LevelBonus) × GradeDamageMultiplier
  - Range = BaseRange × GradeRangeMultiplier
- Reorganize Core folder structure:
  - Units/: Unit, UnitAttack, UnitAbility, UnitUI, UnitDrag, UnitMergeManager, etc.
  - Projectiles/: Bullet, GroundEffect
  - Enemies/: Enemy, PathAgent, Pathfinder
  - Managers/: GameManager, WaveManager, GachaManager, TowerLevelManager, etc.
  - Grid/: GridSystem
</commit_message>
<xml_diff>
--- a/Assets/Data/GameData.xlsx
+++ b/Assets/Data/GameData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\DefenceGame\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18E695DA-5EBB-45EB-9F70-82122E2FAA49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DEA9FCE-3FD3-4623-8AE5-9FE18EAF0455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enemies" sheetId="1" r:id="rId1"/>
@@ -1269,7 +1269,7 @@
         <v>31</v>
       </c>
       <c r="C3">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D3">
         <v>0.8</v>
@@ -1309,7 +1309,7 @@
         <v>13</v>
       </c>
       <c r="C5">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -1329,9 +1329,11 @@
         <v>9</v>
       </c>
       <c r="C6">
+        <f>C2</f>
         <v>10</v>
       </c>
       <c r="D6">
+        <f>D2</f>
         <v>2</v>
       </c>
       <c r="E6">
@@ -1349,9 +1351,11 @@
         <v>31</v>
       </c>
       <c r="C7">
-        <v>25</v>
+        <f t="shared" ref="C7:D21" si="0">C3</f>
+        <v>30</v>
       </c>
       <c r="D7">
+        <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
       <c r="E7">
@@ -1369,9 +1373,11 @@
         <v>32</v>
       </c>
       <c r="C8">
+        <f t="shared" si="0"/>
         <v>50</v>
       </c>
       <c r="D8">
+        <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
       <c r="E8">
@@ -1389,9 +1395,11 @@
         <v>13</v>
       </c>
       <c r="C9">
-        <v>100</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
       <c r="D9">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="E9">
@@ -1409,9 +1417,11 @@
         <v>9</v>
       </c>
       <c r="C10">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="D10">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="E10">
@@ -1429,9 +1439,11 @@
         <v>31</v>
       </c>
       <c r="C11">
-        <v>25</v>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="D11">
+        <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
       <c r="E11">
@@ -1449,9 +1461,11 @@
         <v>32</v>
       </c>
       <c r="C12">
+        <f t="shared" si="0"/>
         <v>50</v>
       </c>
       <c r="D12">
+        <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
       <c r="E12">
@@ -1469,9 +1483,11 @@
         <v>13</v>
       </c>
       <c r="C13">
-        <v>100</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
       <c r="D13">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="E13">
@@ -1489,9 +1505,11 @@
         <v>9</v>
       </c>
       <c r="C14">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="D14">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="E14">
@@ -1509,9 +1527,11 @@
         <v>31</v>
       </c>
       <c r="C15">
-        <v>25</v>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="D15">
+        <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
       <c r="E15">
@@ -1529,9 +1549,11 @@
         <v>32</v>
       </c>
       <c r="C16">
+        <f t="shared" si="0"/>
         <v>50</v>
       </c>
       <c r="D16">
+        <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
       <c r="E16">
@@ -1549,9 +1571,11 @@
         <v>13</v>
       </c>
       <c r="C17">
-        <v>100</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
       <c r="D17">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="E17">
@@ -1569,9 +1593,11 @@
         <v>9</v>
       </c>
       <c r="C18">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="D18">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="E18">
@@ -1589,9 +1615,11 @@
         <v>31</v>
       </c>
       <c r="C19">
-        <v>25</v>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="D19">
+        <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
       <c r="E19">
@@ -1609,9 +1637,11 @@
         <v>32</v>
       </c>
       <c r="C20">
+        <f t="shared" si="0"/>
         <v>50</v>
       </c>
       <c r="D20">
+        <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
       <c r="E20">
@@ -1629,9 +1659,11 @@
         <v>13</v>
       </c>
       <c r="C21">
-        <v>100</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
       <c r="D21">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="E21">
@@ -1684,10 +1716,10 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -1701,10 +1733,10 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D3">
-        <v>1.8</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -1718,7 +1750,7 @@
         <v>2</v>
       </c>
       <c r="C4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -1735,10 +1767,10 @@
         <v>3</v>
       </c>
       <c r="C5">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>0.1</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -1755,7 +1787,7 @@
         <v>5</v>
       </c>
       <c r="D6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -1787,10 +1819,11 @@
       </c>
       <c r="C8">
         <f>INT((PRODUCT(C2,1.5)))</f>
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D8">
-        <v>2</v>
+        <f>D2</f>
+        <v>1</v>
       </c>
       <c r="E8">
         <v>1.2</v>
@@ -1805,10 +1838,11 @@
       </c>
       <c r="C9">
         <f t="shared" ref="C9:C19" si="0">INT((PRODUCT(C3,1.5)))</f>
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="D9">
-        <v>1.8</v>
+        <f t="shared" ref="D9:D19" si="1">D3</f>
+        <v>1</v>
       </c>
       <c r="E9">
         <v>1.2</v>
@@ -1823,9 +1857,10 @@
       </c>
       <c r="C10">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="D10">
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="E10">
@@ -1841,10 +1876,11 @@
       </c>
       <c r="C11">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>150</v>
       </c>
       <c r="D11">
-        <v>2</v>
+        <f t="shared" si="1"/>
+        <v>0.1</v>
       </c>
       <c r="E11">
         <v>1.2</v>
@@ -1862,7 +1898,8 @@
         <v>7</v>
       </c>
       <c r="D12">
-        <v>3</v>
+        <f t="shared" si="1"/>
+        <v>1</v>
       </c>
       <c r="E12">
         <v>1.2</v>
@@ -1880,6 +1917,7 @@
         <v>1</v>
       </c>
       <c r="D13">
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="E13">
@@ -1895,10 +1933,11 @@
       </c>
       <c r="C14">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D14">
-        <v>2</v>
+        <f t="shared" si="1"/>
+        <v>1</v>
       </c>
       <c r="E14">
         <v>1.5</v>
@@ -1913,10 +1952,11 @@
       </c>
       <c r="C15">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="D15">
-        <v>1.8</v>
+        <f t="shared" si="1"/>
+        <v>1</v>
       </c>
       <c r="E15">
         <v>1.5</v>
@@ -1931,9 +1971,10 @@
       </c>
       <c r="C16">
         <f t="shared" si="0"/>
-        <v>67</v>
+        <v>45</v>
       </c>
       <c r="D16">
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="E16">
@@ -1949,10 +1990,11 @@
       </c>
       <c r="C17">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>225</v>
       </c>
       <c r="D17">
-        <v>2</v>
+        <f t="shared" si="1"/>
+        <v>0.1</v>
       </c>
       <c r="E17">
         <v>1.5</v>
@@ -1970,7 +2012,8 @@
         <v>10</v>
       </c>
       <c r="D18">
-        <v>3</v>
+        <f t="shared" si="1"/>
+        <v>1</v>
       </c>
       <c r="E18">
         <v>1.5</v>
@@ -1988,6 +2031,7 @@
         <v>1</v>
       </c>
       <c r="D19">
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="E19">
@@ -2111,7 +2155,7 @@
         <v>1.5</v>
       </c>
       <c r="C3">
-        <v>1.2</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="D3">
         <v>1.1000000000000001</v>
@@ -2125,7 +2169,7 @@
         <v>2</v>
       </c>
       <c r="C4">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="D4">
         <v>1.3</v>
@@ -2139,7 +2183,7 @@
         <v>2.5</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="D5">
         <v>1.5</v>
@@ -2153,7 +2197,7 @@
         <v>5</v>
       </c>
       <c r="C6">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="D6">
         <v>2</v>

</xml_diff>

<commit_message>
fix: Bullet/GroundEffect collision detection and range calculation
- Bullet.cs: Add Rigidbody2D and CircleCollider2D in Awake for proper OnTriggerEnter2D detection
- GroundEffect.cs: Simplify damage detection using OnTriggerEnter2D/OnTriggerExit2D
- Unit.cs: Reduce range calculation by dividing by 2.5 (too large, minimum was 8, now ~3.2)
</commit_message>
<xml_diff>
--- a/Assets/Data/GameData.xlsx
+++ b/Assets/Data/GameData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\DefenceGame\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DEA9FCE-3FD3-4623-8AE5-9FE18EAF0455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A8A99FB-88CE-447D-85AD-9DA03EB70703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enemies" sheetId="1" r:id="rId1"/>
@@ -1255,7 +1255,7 @@
         <v>2</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
@@ -1275,7 +1275,7 @@
         <v>0.8</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F3" t="s">
         <v>10</v>
@@ -1295,7 +1295,7 @@
         <v>0.8</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" t="s">
         <v>10</v>
@@ -1315,7 +1315,7 @@
         <v>1</v>
       </c>
       <c r="E5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5" t="s">
         <v>10</v>
@@ -1337,7 +1337,7 @@
         <v>2</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F6" t="s">
         <v>30</v>
@@ -1359,7 +1359,7 @@
         <v>0.8</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F7" t="s">
         <v>30</v>
@@ -1381,7 +1381,7 @@
         <v>0.8</v>
       </c>
       <c r="E8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F8" t="s">
         <v>30</v>
@@ -1403,7 +1403,7 @@
         <v>1</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" t="s">
         <v>30</v>
@@ -1425,7 +1425,7 @@
         <v>2</v>
       </c>
       <c r="E10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F10" t="s">
         <v>29</v>
@@ -1447,7 +1447,7 @@
         <v>0.8</v>
       </c>
       <c r="E11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F11" t="s">
         <v>29</v>
@@ -1469,7 +1469,7 @@
         <v>0.8</v>
       </c>
       <c r="E12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" t="s">
         <v>29</v>
@@ -1491,7 +1491,7 @@
         <v>1</v>
       </c>
       <c r="E13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F13" t="s">
         <v>29</v>
@@ -1513,7 +1513,7 @@
         <v>2</v>
       </c>
       <c r="E14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F14" t="s">
         <v>12</v>
@@ -1535,7 +1535,7 @@
         <v>0.8</v>
       </c>
       <c r="E15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F15" t="s">
         <v>12</v>
@@ -1557,7 +1557,7 @@
         <v>0.8</v>
       </c>
       <c r="E16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F16" t="s">
         <v>12</v>
@@ -1579,7 +1579,7 @@
         <v>1</v>
       </c>
       <c r="E17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F17" t="s">
         <v>12</v>
@@ -1601,7 +1601,7 @@
         <v>2</v>
       </c>
       <c r="E18">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F18" t="s">
         <v>14</v>
@@ -1623,7 +1623,7 @@
         <v>0.8</v>
       </c>
       <c r="E19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F19" t="s">
         <v>14</v>
@@ -1645,7 +1645,7 @@
         <v>0.8</v>
       </c>
       <c r="E20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F20" t="s">
         <v>14</v>
@@ -1667,7 +1667,7 @@
         <v>1</v>
       </c>
       <c r="E21">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F21" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
refactor: Remove test code and Debug.Logs
- Delete GradeAbilityTestManager.cs (test manager for grade-based abilities)
- Remove test mode from UnitAbility.cs (autoApplyCurrentLevel, ForceApplyLevel)
- Remove all Debug.Log statements from UnitAbility.cs
- Remove Debug.Log from Unit.cs Initialize method
- Remove test click buttons from TowerLevelUI.cs (SetupClickButtons, OnSlotClicked)
</commit_message>
<xml_diff>
--- a/Assets/Data/GameData.xlsx
+++ b/Assets/Data/GameData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\DefenceGame\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A8A99FB-88CE-447D-85AD-9DA03EB70703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6BAAD45-8B61-48ED-A0F9-407DFD5BCB53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1255,7 +1255,7 @@
         <v>2</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
@@ -1275,7 +1275,7 @@
         <v>0.8</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F3" t="s">
         <v>10</v>
@@ -1295,7 +1295,7 @@
         <v>0.8</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F4" t="s">
         <v>10</v>
@@ -1315,7 +1315,7 @@
         <v>1</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F5" t="s">
         <v>10</v>
@@ -1337,7 +1337,7 @@
         <v>2</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F6" t="s">
         <v>30</v>
@@ -1359,7 +1359,7 @@
         <v>0.8</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F7" t="s">
         <v>30</v>
@@ -1381,7 +1381,7 @@
         <v>0.8</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F8" t="s">
         <v>30</v>
@@ -1403,7 +1403,7 @@
         <v>1</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9" t="s">
         <v>30</v>
@@ -1425,7 +1425,7 @@
         <v>2</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F10" t="s">
         <v>29</v>
@@ -1447,7 +1447,7 @@
         <v>0.8</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F11" t="s">
         <v>29</v>
@@ -1469,7 +1469,7 @@
         <v>0.8</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F12" t="s">
         <v>29</v>
@@ -1491,7 +1491,7 @@
         <v>1</v>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F13" t="s">
         <v>29</v>
@@ -1513,7 +1513,7 @@
         <v>2</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F14" t="s">
         <v>12</v>
@@ -1535,7 +1535,7 @@
         <v>0.8</v>
       </c>
       <c r="E15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F15" t="s">
         <v>12</v>
@@ -1557,7 +1557,7 @@
         <v>0.8</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F16" t="s">
         <v>12</v>
@@ -1579,7 +1579,7 @@
         <v>1</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F17" t="s">
         <v>12</v>
@@ -1601,7 +1601,7 @@
         <v>2</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F18" t="s">
         <v>14</v>
@@ -1623,7 +1623,7 @@
         <v>0.8</v>
       </c>
       <c r="E19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F19" t="s">
         <v>14</v>
@@ -1645,7 +1645,7 @@
         <v>0.8</v>
       </c>
       <c r="E20">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F20" t="s">
         <v>14</v>
@@ -1667,7 +1667,7 @@
         <v>1</v>
       </c>
       <c r="E21">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F21" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
feat: Add enemy kill exp system and fix merge color bug
1. Fix: Unit rare color not changing on merge
   - Add unitUI.SetGradeColor call in Unit.Initialize

2. Add enemy kill exp system
   - Enemy.cs: Add lastAttacker tracking
   - Enemy.cs: Add TakeDamage(Unit attacker) overload
   - TowerLevelManager.cs: Add AddExpFromKill method
   - Bullet.cs: Add attacker field and pass to enemies
   - UnitAttack.cs: Pass unit as attacker in all attack methods

3. Field unit level up system (already working)
   - Unit.cs subscribes to TowerLevelUp event
   - UnitAbility.OnLevelUp applies level abilities automatically

4. Gacha spawn with current tower level
   - UnitAbility.Initialize already gets current level from TowerLevelManager
</commit_message>
<xml_diff>
--- a/Assets/Data/GameData.xlsx
+++ b/Assets/Data/GameData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\DefenceGame\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6BAAD45-8B61-48ED-A0F9-407DFD5BCB53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CB755AB-1CDE-42FF-AAD7-967F864A6024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enemies" sheetId="1" r:id="rId1"/>
@@ -58,9 +58,6 @@
     <t>AttackSpeed</t>
   </si>
   <si>
-    <t>Range</t>
-  </si>
-  <si>
     <t>Grade</t>
   </si>
   <si>
@@ -98,9 +95,6 @@
   </si>
   <si>
     <t>DamageMultiplier</t>
-  </si>
-  <si>
-    <t>RangeMultiplier</t>
   </si>
   <si>
     <t>BlackSlime</t>
@@ -144,6 +138,14 @@
   </si>
   <si>
     <t>WizardTower</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Range</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>RangeMultiplier</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1125,7 +1127,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C2">
         <v>30</v>
@@ -1142,7 +1144,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C3">
         <v>50</v>
@@ -1159,7 +1161,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C4">
         <v>20</v>
@@ -1176,7 +1178,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -1193,7 +1195,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C6">
         <v>1000</v>
@@ -1235,10 +1237,10 @@
         <v>6</v>
       </c>
       <c r="E1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" t="s">
         <v>7</v>
-      </c>
-      <c r="F1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1246,7 +1248,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C2">
         <v>10</v>
@@ -1258,7 +1260,7 @@
         <v>3</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -1266,7 +1268,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C3">
         <v>30</v>
@@ -1278,7 +1280,7 @@
         <v>3</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -1286,7 +1288,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C4">
         <v>50</v>
@@ -1298,7 +1300,7 @@
         <v>3</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -1306,7 +1308,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5">
         <v>50</v>
@@ -1318,7 +1320,7 @@
         <v>3</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -1326,7 +1328,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6">
         <f>C2</f>
@@ -1340,7 +1342,7 @@
         <v>3</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -1348,7 +1350,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C7">
         <f t="shared" ref="C7:D21" si="0">C3</f>
@@ -1362,7 +1364,7 @@
         <v>3</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -1370,7 +1372,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C8">
         <f t="shared" si="0"/>
@@ -1384,7 +1386,7 @@
         <v>3</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -1392,7 +1394,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
@@ -1406,7 +1408,7 @@
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -1414,7 +1416,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C10">
         <f t="shared" si="0"/>
@@ -1428,7 +1430,7 @@
         <v>3</v>
       </c>
       <c r="F10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -1436,7 +1438,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C11">
         <f t="shared" si="0"/>
@@ -1450,7 +1452,7 @@
         <v>3</v>
       </c>
       <c r="F11" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -1458,7 +1460,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C12">
         <f t="shared" si="0"/>
@@ -1472,7 +1474,7 @@
         <v>3</v>
       </c>
       <c r="F12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -1480,7 +1482,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C13">
         <f t="shared" si="0"/>
@@ -1494,7 +1496,7 @@
         <v>3</v>
       </c>
       <c r="F13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -1502,7 +1504,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C14">
         <f t="shared" si="0"/>
@@ -1516,7 +1518,7 @@
         <v>3</v>
       </c>
       <c r="F14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -1524,7 +1526,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C15">
         <f t="shared" si="0"/>
@@ -1538,7 +1540,7 @@
         <v>3</v>
       </c>
       <c r="F15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -1546,7 +1548,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C16">
         <f t="shared" si="0"/>
@@ -1560,7 +1562,7 @@
         <v>3</v>
       </c>
       <c r="F16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -1568,7 +1570,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C17">
         <f t="shared" si="0"/>
@@ -1582,7 +1584,7 @@
         <v>3</v>
       </c>
       <c r="F17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -1590,7 +1592,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C18">
         <f t="shared" si="0"/>
@@ -1604,7 +1606,7 @@
         <v>3</v>
       </c>
       <c r="F18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -1612,7 +1614,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C19">
         <f t="shared" si="0"/>
@@ -1626,7 +1628,7 @@
         <v>3</v>
       </c>
       <c r="F19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -1634,7 +1636,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C20">
         <f t="shared" si="0"/>
@@ -1648,7 +1650,7 @@
         <v>3</v>
       </c>
       <c r="F20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -1656,21 +1658,21 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="D21">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <v>3</v>
+      </c>
+      <c r="F21" t="s">
         <v>13</v>
-      </c>
-      <c r="C21">
-        <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-      <c r="D21">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="E21">
-        <v>3</v>
-      </c>
-      <c r="F21" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1693,19 +1695,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
         <v>15</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>17</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>18</v>
-      </c>
-      <c r="E1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -2055,15 +2057,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2">
         <f>100-SUM(B3:B6)</f>
@@ -2072,7 +2074,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B3">
         <v>15</v>
@@ -2080,7 +2082,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>6</v>
@@ -2088,7 +2090,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>3</v>
@@ -2096,7 +2098,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -2121,27 +2123,27 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C1" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -2149,13 +2151,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
       <c r="C3">
-        <v>1.1000000000000001</v>
+        <v>0.9</v>
       </c>
       <c r="D3">
         <v>1.1000000000000001</v>
@@ -2163,44 +2165,44 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>2</v>
       </c>
       <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
         <v>1.2</v>
-      </c>
-      <c r="D4">
-        <v>1.3</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>2.5</v>
       </c>
       <c r="C5">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D5">
         <v>1.3</v>
-      </c>
-      <c r="D5">
-        <v>1.5</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6">
         <v>5</v>
       </c>
       <c r="C6">
+        <v>1.2</v>
+      </c>
+      <c r="D6">
         <v>1.5</v>
-      </c>
-      <c r="D6">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Set starting gold to 200
</commit_message>
<xml_diff>
--- a/Assets/Data/GameData.xlsx
+++ b/Assets/Data/GameData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\DefenceGame\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CB755AB-1CDE-42FF-AAD7-967F864A6024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F696DD43-C4E4-45D2-8CA8-63BB9A3C9632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enemies" sheetId="1" r:id="rId1"/>
@@ -1251,7 +1251,7 @@
         <v>8</v>
       </c>
       <c r="C2">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D2">
         <v>2</v>
@@ -1274,7 +1274,7 @@
         <v>30</v>
       </c>
       <c r="D3">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -1294,7 +1294,7 @@
         <v>50</v>
       </c>
       <c r="D4">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -1311,10 +1311,10 @@
         <v>12</v>
       </c>
       <c r="C5">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E5">
         <v>3</v>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="C6">
         <f>C2</f>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D6">
         <f>D2</f>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="D7">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E7">
         <v>3</v>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="D8">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E8">
         <v>3</v>
@@ -1398,11 +1398,11 @@
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="D9">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E9">
         <v>3</v>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="C10">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D10">
         <f t="shared" si="0"/>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D11">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E11">
         <v>3</v>
@@ -1468,7 +1468,7 @@
       </c>
       <c r="D12">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E12">
         <v>3</v>
@@ -1486,11 +1486,11 @@
       </c>
       <c r="C13">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="D13">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E13">
         <v>3</v>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="C14">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D14">
         <f t="shared" si="0"/>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="D15">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E15">
         <v>3</v>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="D16">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E16">
         <v>3</v>
@@ -1574,11 +1574,11 @@
       </c>
       <c r="C17">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="D17">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E17">
         <v>3</v>
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C18">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D18">
         <f t="shared" si="0"/>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="D19">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E19">
         <v>3</v>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="D20">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E20">
         <v>3</v>
@@ -1662,11 +1662,11 @@
       </c>
       <c r="C21">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="D21">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E21">
         <v>3</v>
@@ -2154,7 +2154,7 @@
         <v>28</v>
       </c>
       <c r="B3">
-        <v>1.5</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="C3">
         <v>0.9</v>
@@ -2168,7 +2168,7 @@
         <v>10</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -2182,7 +2182,7 @@
         <v>11</v>
       </c>
       <c r="B5">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="C5">
         <v>1.1000000000000001</v>
@@ -2196,7 +2196,7 @@
         <v>13</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C6">
         <v>1.2</v>

</xml_diff>

<commit_message>
feat: Wait for boss death before next wave
- WaveManager now tracks current boss
- Boss wave (wave 6, 12, 18...) waits until boss is defeated
- Added isBossWave and currentBoss fields
- Modified SpawnEnemy to return Enemy for tracking
- Next wave only starts after boss death + 3s delay
</commit_message>
<xml_diff>
--- a/Assets/Data/GameData.xlsx
+++ b/Assets/Data/GameData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\DefenceGame\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89DB9EB9-0A69-446C-8B34-FDBF014892E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{073D4729-4EFF-4673-B37C-099D1D7B1ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4200" yWindow="1365" windowWidth="21600" windowHeight="11385" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1721,7 +1721,7 @@
         <v>15</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -1738,7 +1738,7 @@
         <v>20</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -1755,7 +1755,7 @@
         <v>20</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -1789,7 +1789,7 @@
         <v>10</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E6">
         <v>1</v>

</xml_diff>